<commit_message>
fix(booking): add try-catch error handling to saveAsTemplate and onPromptConfirm
</commit_message>
<xml_diff>
--- a/docs/imp.xlsx
+++ b/docs/imp.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30048" windowHeight="13740" tabRatio="873" activeTab="6"/>
+    <workbookView windowWidth="20783" windowHeight="12048" tabRatio="873" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="2026.01" sheetId="2" r:id="rId1"/>
@@ -13132,8 +13132,7 @@
   <cols>
     <col min="1" max="1" width="11.5092592592593" style="6" customWidth="1"/>
     <col min="2" max="2" width="19.5092592592593" style="6" customWidth="1"/>
-    <col min="3" max="3" width="11.5092592592593" style="6" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5092592592593" style="6" customWidth="1"/>
+    <col min="3" max="4" width="11.5092592592593" style="6" customWidth="1"/>
     <col min="5" max="5" width="23.5092592592593" style="6" customWidth="1"/>
     <col min="6" max="16384" width="9" style="6"/>
   </cols>

</xml_diff>